<commit_message>
Kit WLDBNT : dès 9 ans, jaquette, 295 g
</commit_message>
<xml_diff>
--- a/wldbntT1-T2_kit/fiche-technique-matrice.xlsx
+++ b/wldbntT1-T2_kit/fiche-technique-matrice.xlsx
@@ -1592,7 +1592,9 @@
       <c r="S2" s="91" t="n">
         <v>210</v>
       </c>
-      <c r="T2" s="91" t="n"/>
+      <c r="T2" s="91" t="n">
+        <v>295</v>
+      </c>
       <c r="U2" s="97" t="n">
         <v>45566</v>
       </c>
@@ -1626,7 +1628,7 @@
       <c r="AC2" s="91" t="n"/>
       <c r="AD2" s="91" t="inlineStr">
         <is>
-          <t>de 9 à 14 ans</t>
+          <t>à partir de 9 ans</t>
         </is>
       </c>
       <c r="AE2" s="98" t="n">
@@ -1634,7 +1636,7 @@
       </c>
       <c r="AF2" s="91" t="inlineStr">
         <is>
-          <t>Walad et Binti remplacent Tonton aux commandes de Foulanville 3.0, la ville virtuelle attaquée par les Pirates. Manga, 9-14 ans.</t>
+          <t>Walad et Binti remplacent Tonton aux commandes de Foulanville 3.0, la ville virtuelle attaquée par les Pirates. Manga, dès 9 ans.</t>
         </is>
       </c>
       <c r="AG2" s="91" t="n"/>
@@ -1721,7 +1723,9 @@
       <c r="S3" s="91" t="n">
         <v>210</v>
       </c>
-      <c r="T3" s="91" t="n"/>
+      <c r="T3" s="91" t="n">
+        <v>295</v>
+      </c>
       <c r="U3" s="99" t="n">
         <v>46143</v>
       </c>
@@ -1755,7 +1759,7 @@
       <c r="AC3" s="91" t="n"/>
       <c r="AD3" s="91" t="inlineStr">
         <is>
-          <t>de 9 à 14 ans</t>
+          <t>à partir de 9 ans</t>
         </is>
       </c>
       <c r="AE3" s="98" t="n">
@@ -1763,7 +1767,7 @@
       </c>
       <c r="AF3" s="91" t="inlineStr">
         <is>
-          <t>Les Bannis prennent Oldtown et piègent les habitants avec une arnaque au clic. La suite directe du tome 1. Manga, 9-14 ans.</t>
+          <t>Les Bannis prennent Oldtown et piègent les habitants avec une arnaque au clic. La suite directe du tome 1. Manga, dès 9 ans.</t>
         </is>
       </c>
       <c r="AG3" s="91" t="n"/>

</xml_diff>

<commit_message>
Kit WLDBNT : 300 g, parution = 1re vente
</commit_message>
<xml_diff>
--- a/wldbntT1-T2_kit/fiche-technique-matrice.xlsx
+++ b/wldbntT1-T2_kit/fiche-technique-matrice.xlsx
@@ -1593,10 +1593,10 @@
         <v>210</v>
       </c>
       <c r="T2" s="91" t="n">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="U2" s="97" t="n">
-        <v>45566</v>
+        <v>45586</v>
       </c>
       <c r="V2" s="91" t="inlineStr">
         <is>
@@ -1724,10 +1724,10 @@
         <v>210</v>
       </c>
       <c r="T3" s="91" t="n">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="U3" s="99" t="n">
-        <v>46143</v>
+        <v>46146</v>
       </c>
       <c r="V3" s="91" t="inlineStr">
         <is>

</xml_diff>